<commit_message>
Refresh pillar 3 maintainer drift docs
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$14</definedName>

</xml_diff>

<commit_message>
Refresh pillar 4 maintainer drift docs
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$14</definedName>

</xml_diff>

<commit_message>
Fix pillar 3 priority cleanup drift
Align the recommended retention tier with the current Priority cleanup scope
and regenerate checklist templates from the repo generator.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$14</definedName>

</xml_diff>

<commit_message>
fix: reconcile manifest control role ownership
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8.0  |  10 controls</t>
+          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8.0  |  12 controls</t>
         </is>
       </c>
     </row>
@@ -724,17 +724,17 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3.8a</t>
+          <t>2.17</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
+          <t>Cross-Tenant Agent Federation (MCP and Entra Agent ID)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>P3 – Compliance &amp; Records</t>
+          <t>P2 – Security &amp; Data Protection</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -744,17 +744,17 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
+          <t>Copilot Chat; Pages; Agents; Purview DLP/Labels</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Has a generative-AI model-governance review (NIST AI RMF 1.0 / ISO/IEC 42001, addressing the SR 26-2 / OCC 2026-13 generative-AI exclusion) been completed for Copilot?</t>
+          <t>Are cross-tenant Entra Agent ID trust relationships, MCP federated server attestations, and Copilot Studio multi-tenant publishings subject to documented approval and review?</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Generative-AI governance review document for Copilot; NIST AI RMF 1.0 alignment documentation; Bias testing and safety evaluation results; Responsible-AI principles adoption evidence</t>
+          <t>Cross-tenant trust relationship inventory with named owners; Approval records for each trust relationship; MCP federated server attestation documentation; Periodic review cadence and most recent review date</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
@@ -763,12 +763,12 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.8a</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>FFIEC IT Examination Handbook Alignment</t>
+          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
+          <t>Has a generative-AI model-governance review (NIST AI RMF 1.0 / ISO/IEC 42001, addressing the SR 26-2 / OCC 2026-13 generative-AI exclusion) been completed for Copilot?</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
+          <t>Generative-AI governance review document for Copilot; NIST AI RMF 1.0 alignment documentation; Bias testing and safety evaluation results; Responsible-AI principles adoption evidence</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -802,17 +802,17 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
+          <t>FFIEC IT Examination Handbook Alignment</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>P4 – Operations &amp; Lifecycle</t>
+          <t>P3 – Compliance &amp; Records</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Are Viva Insights Copilot impact reports reviewed on a documented cadence with caveats applied?</t>
+          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
+          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
@@ -841,12 +841,12 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Copilot Extensibility and Agent Operations Governance</t>
+          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Are extensibility surfaces (declarative agents, MCP, plug-ins) governed by an approval and inventory process before publication?</t>
+          <t>Are Viva Insights Copilot impact reports reviewed on a documented cadence with caveats applied?</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
+          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -880,12 +880,12 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Copilot Cowork Governance</t>
+          <t>Copilot Extensibility and Agent Operations Governance</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
+          <t>Are extensibility surfaces (declarative agents, MCP, plug-ins) governed by an approval and inventory process before publication?</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
@@ -919,12 +919,12 @@
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Scout Governance</t>
+          <t>Copilot Studio Agent Lifecycle Governance</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -944,25 +944,103 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+          <t>Is the Copilot Studio agent lifecycle (authoring → testing → publishing → versioning → deprecation) governed with documented evidence at each gate?</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+          <t>Agent lifecycle governance policy document; Lifecycle gate evidence (testing, approval, publishing records); Agent inventory with lifecycle stage tracking; Retirement/deprecation documentation for decommissioned agents</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
       <c r="I14" s="7" t="inlineStr"/>
     </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>4.15</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Copilot Cowork Governance</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Scout Governance</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I14"/>
+  <autoFilter ref="A4:I16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: reconcile manifest control role ownership (#537)
* fix: reconcile manifest control role ownership

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

* chore: refresh PR 537 on main

Merge origin/main and confirm generated manifest/checklist outputs are clean after regeneration.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

---------

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8.0  |  10 controls</t>
+          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8.0  |  12 controls</t>
         </is>
       </c>
     </row>
@@ -724,17 +724,17 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3.8a</t>
+          <t>2.17</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
+          <t>Cross-Tenant Agent Federation (MCP and Entra Agent ID)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>P3 – Compliance &amp; Records</t>
+          <t>P2 – Security &amp; Data Protection</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -744,17 +744,17 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
+          <t>Copilot Chat; Pages; Agents; Purview DLP/Labels</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Has a generative-AI model-governance review (NIST AI RMF 1.0 / ISO/IEC 42001, addressing the SR 26-2 / OCC 2026-13 generative-AI exclusion) been completed for Copilot?</t>
+          <t>Are cross-tenant Entra Agent ID trust relationships, MCP federated server attestations, and Copilot Studio multi-tenant publishings subject to documented approval and review?</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Generative-AI governance review document for Copilot; NIST AI RMF 1.0 alignment documentation; Bias testing and safety evaluation results; Responsible-AI principles adoption evidence</t>
+          <t>Cross-tenant trust relationship inventory with named owners; Approval records for each trust relationship; MCP federated server attestation documentation; Periodic review cadence and most recent review date</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
@@ -763,12 +763,12 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.8a</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>FFIEC IT Examination Handbook Alignment</t>
+          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -788,12 +788,12 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
+          <t>Has a generative-AI model-governance review (NIST AI RMF 1.0 / ISO/IEC 42001, addressing the SR 26-2 / OCC 2026-13 generative-AI exclusion) been completed for Copilot?</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
+          <t>Generative-AI governance review document for Copilot; NIST AI RMF 1.0 alignment documentation; Bias testing and safety evaluation results; Responsible-AI principles adoption evidence</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -802,17 +802,17 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
+          <t>FFIEC IT Examination Handbook Alignment</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>P4 – Operations &amp; Lifecycle</t>
+          <t>P3 – Compliance &amp; Records</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -822,17 +822,17 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Are Viva Insights Copilot impact reports reviewed on a documented cadence with caveats applied?</t>
+          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
+          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
@@ -841,12 +841,12 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Copilot Extensibility and Agent Operations Governance</t>
+          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Are extensibility surfaces (declarative agents, MCP, plug-ins) governed by an approval and inventory process before publication?</t>
+          <t>Are Viva Insights Copilot impact reports reviewed on a documented cadence with caveats applied?</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
+          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -880,12 +880,12 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Copilot Cowork Governance</t>
+          <t>Copilot Extensibility and Agent Operations Governance</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
+          <t>Are extensibility surfaces (declarative agents, MCP, plug-ins) governed by an approval and inventory process before publication?</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
@@ -919,12 +919,12 @@
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Scout Governance</t>
+          <t>Copilot Studio Agent Lifecycle Governance</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -944,25 +944,103 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+          <t>Is the Copilot Studio agent lifecycle (authoring → testing → publishing → versioning → deprecation) governed with documented evidence at each gate?</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+          <t>Agent lifecycle governance policy document; Lifecycle gate evidence (testing, approval, publishing records); Agent inventory with lifecycle stage tracking; Retirement/deprecation documentation for decommissioned agents</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
       <c r="I14" s="7" t="inlineStr"/>
     </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>4.15</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Copilot Cowork Governance</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Scout Governance</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I14"/>
+  <autoFilter ref="A4:I16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore: regenerate control content graph
Regenerate the canonical content graph after the 1.1, 1.11, and 1.12 Last Verified updates.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$16</definedName>

</xml_diff>

<commit_message>
docs: refresh Cowork and usage-based billing guidance
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$16</definedName>
@@ -988,7 +988,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+          <t>Usage-based billing scope export (user/group assignments) with approver; Current discovery-setting decision record, transition note, and access-request workflow evidence; Model-policy record for Anthropic family and any enabled provider-retention model variants; Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy plus recent Cost management and Cowork usage reports; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: refresh Cowork and usage-based billing guidance (#564)
Part of the documentation freshness program.
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$16</definedName>
@@ -988,7 +988,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+          <t>Usage-based billing scope export (user/group assignments) with approver; Current discovery-setting decision record, transition note, and access-request workflow evidence; Model-policy record for Anthropic family and any enabled provider-retention model variants; Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy plus recent Cost management and Cowork usage reports; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>

</xml_diff>